<commit_message>
file clean up and changes to injury names/codes
</commit_message>
<xml_diff>
--- a/myCBD/myInfo/gbd.ICD.Map.xlsx
+++ b/myCBD/myInfo/gbd.ICD.Map.xlsx
@@ -113,7 +113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2869" uniqueCount="1403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2869" uniqueCount="1402">
   <si>
     <t>I. Communicable, maternal, perinatal and nutritional conditions</t>
   </si>
@@ -3533,9 +3533,6 @@
   </si>
   <si>
     <t>b</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
   <si>
     <t>Other Infectious Diseases</t>
@@ -4195,9 +4192,6 @@
     <t xml:space="preserve">J. Digestive diseases </t>
   </si>
   <si>
-    <t>INCLUDED FOR NOW WITH UNINTENTIONAL -- FIX</t>
-  </si>
-  <si>
     <t>E10[0-1,3-9]|E11[0-1,3-9]|E12[0-1,3-9]|E13[0-1,3-9]|E14[0-1,3-9]|R730|R739</t>
   </si>
   <si>
@@ -4470,6 +4464,9 @@
   </si>
   <si>
     <t>Poisonings (non-substance use)</t>
+  </si>
+  <si>
+    <t>INCLUDED ALL INJURY but not elsewhere</t>
   </si>
 </sst>
 </file>
@@ -4651,7 +4648,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4721,6 +4718,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4804,7 +4807,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -5062,6 +5065,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="29">
@@ -5427,7 +5433,7 @@
   <sheetData>
     <row r="1" spans="1:24" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>761</v>
@@ -5436,7 +5442,7 @@
         <v>763</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="E1" s="24" t="s">
         <v>1121</v>
@@ -5451,10 +5457,10 @@
         <v>1124</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>384</v>
@@ -5463,19 +5469,19 @@
         <v>759</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
       <c r="O1" s="59" t="s">
+        <v>1160</v>
+      </c>
+      <c r="P1" s="59" t="s">
         <v>1161</v>
       </c>
-      <c r="P1" s="59" t="s">
-        <v>1162</v>
-      </c>
       <c r="Q1" s="59" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="R1" s="82" t="s">
         <v>509</v>
@@ -5490,10 +5496,10 @@
         <v>762</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="W1" s="45" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="X1" s="6" t="s">
         <v>930</v>
@@ -5557,7 +5563,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E3" s="26"/>
       <c r="F3" s="6"/>
@@ -5606,10 +5612,10 @@
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="29" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E4" s="26">
         <v>99</v>
@@ -5632,11 +5638,11 @@
       <c r="R4" s="83"/>
       <c r="S4" s="83"/>
       <c r="T4" s="20" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="U4" s="20"/>
       <c r="V4" s="3" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="W4" s="45"/>
       <c r="X4" s="2"/>
@@ -5704,10 +5710,10 @@
         <v>2</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="40" t="str">
@@ -5763,10 +5769,10 @@
         <v>1125</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="40"/>
@@ -5786,11 +5792,11 @@
       <c r="R7" s="83"/>
       <c r="S7" s="83"/>
       <c r="T7" s="2" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="U7" s="20"/>
       <c r="V7" s="2" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="W7" s="45"/>
       <c r="X7" s="2"/>
@@ -5804,13 +5810,13 @@
         <v>4</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>1126</v>
@@ -5871,10 +5877,10 @@
         <v>4</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>1126</v>
@@ -5931,10 +5937,10 @@
         <v>5</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E10" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>1126</v>
@@ -5991,10 +5997,10 @@
         <v>6</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>1126</v>
@@ -6051,10 +6057,10 @@
         <v>7</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E12" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>1126</v>
@@ -6109,10 +6115,10 @@
         <v>8</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>1126</v>
@@ -6166,13 +6172,13 @@
         <v>10</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>1127</v>
@@ -6231,10 +6237,10 @@
         <v>686</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E15" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>1127</v>
@@ -6287,10 +6293,10 @@
         <v>687</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E16" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>1127</v>
@@ -6347,7 +6353,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E17" s="26">
         <v>99</v>
@@ -6457,7 +6463,7 @@
         <v>12</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E19" s="26">
         <v>99</v>
@@ -6515,7 +6521,7 @@
         <v>13</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E20" s="26">
         <v>99</v>
@@ -6573,7 +6579,7 @@
         <v>14</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E21" s="26">
         <v>99</v>
@@ -6631,7 +6637,7 @@
         <v>15</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E22" s="26">
         <v>99</v>
@@ -6689,10 +6695,10 @@
         <v>16</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="40" t="str">
@@ -6750,10 +6756,10 @@
         <v>17</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="40" t="str">
@@ -6811,10 +6817,10 @@
         <v>688</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="40"/>
@@ -6865,10 +6871,10 @@
         <v>689</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="40" t="str">
@@ -6919,10 +6925,10 @@
         <v>690</v>
       </c>
       <c r="D27" s="27" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>1126</v>
@@ -6973,7 +6979,7 @@
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="34" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="D28" s="27"/>
       <c r="E28" s="26"/>
@@ -7006,10 +7012,10 @@
         <v>691</v>
       </c>
       <c r="D29" s="27" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>1127</v>
@@ -7065,10 +7071,10 @@
         <v>692</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E30" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="40" t="str">
@@ -7170,7 +7176,7 @@
         <v>18</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E32" s="26">
         <v>99</v>
@@ -7228,7 +7234,7 @@
         <v>19</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E33" s="26">
         <v>99</v>
@@ -7286,7 +7292,7 @@
         <v>20</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E34" s="26">
         <v>99</v>
@@ -7344,7 +7350,7 @@
         <v>21</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E35" s="26">
         <v>99</v>
@@ -7402,7 +7408,7 @@
         <v>22</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E36" s="26">
         <v>99</v>
@@ -7460,7 +7466,7 @@
         <v>23</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E37" s="26">
         <v>99</v>
@@ -7514,7 +7520,7 @@
         <v>24</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E38" s="26">
         <v>99</v>
@@ -7568,7 +7574,7 @@
         <v>694</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E39" s="26">
         <v>99</v>
@@ -7626,7 +7632,7 @@
         <v>695</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E40" s="26">
         <v>99</v>
@@ -7684,7 +7690,7 @@
         <v>889</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E41" s="26">
         <v>99</v>
@@ -7738,7 +7744,7 @@
         <v>890</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E42" s="26">
         <v>99</v>
@@ -7796,7 +7802,7 @@
         <v>891</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E43" s="26">
         <v>99</v>
@@ -7850,7 +7856,7 @@
         <v>893</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E44" s="26">
         <v>99</v>
@@ -7908,7 +7914,7 @@
         <v>894</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E45" s="26">
         <v>99</v>
@@ -8021,7 +8027,7 @@
         <v>25</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E47" s="26">
         <v>99</v>
@@ -8079,7 +8085,7 @@
         <v>26</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E48" s="26">
         <v>99</v>
@@ -8133,7 +8139,7 @@
         <v>27</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E49" s="26">
         <v>99</v>
@@ -8187,7 +8193,7 @@
         <v>696</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E50" s="26">
         <v>99</v>
@@ -8241,7 +8247,7 @@
         <v>880</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E51" s="26">
         <v>99</v>
@@ -8253,16 +8259,16 @@
       </c>
       <c r="H51" s="40"/>
       <c r="I51" s="5" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="K51" s="5" t="s">
+        <v>1229</v>
+      </c>
+      <c r="L51" s="19" t="s">
         <v>1230</v>
-      </c>
-      <c r="L51" s="19" t="s">
-        <v>1231</v>
       </c>
       <c r="M51" s="19"/>
       <c r="N51" s="19"/>
@@ -8292,7 +8298,7 @@
         <v>880</v>
       </c>
       <c r="X51" s="5" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="52" spans="1:24" x14ac:dyDescent="0.25">
@@ -8307,10 +8313,10 @@
         <v>28</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E52" s="26" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="40"/>
@@ -8367,10 +8373,10 @@
         <v>29</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E53" s="26" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>1126</v>
@@ -8389,13 +8395,13 @@
         <v>404</v>
       </c>
       <c r="L53" s="75" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="M53" s="75" t="s">
-        <v>1354</v>
+        <v>1352</v>
       </c>
       <c r="N53" s="75" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="O53" s="59" t="s">
         <v>404</v>
@@ -8436,10 +8442,10 @@
         <v>30</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E54" s="26" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>1127</v>
@@ -8505,10 +8511,10 @@
         <v>31</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E55" s="26" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="F55" s="6"/>
       <c r="G55" s="40" t="str">
@@ -8569,10 +8575,10 @@
         <v>32</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E56" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="40" t="s">
@@ -8631,10 +8637,10 @@
         <v>33</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E57" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F57" s="6"/>
       <c r="G57" s="40" t="str">
@@ -8645,16 +8651,16 @@
       <c r="I57" s="5"/>
       <c r="J57" s="5"/>
       <c r="K57" s="5" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="L57" s="16" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="M57" s="16" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
       <c r="N57" s="16" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="O57" s="59" t="s">
         <v>408</v>
@@ -8682,7 +8688,7 @@
         <v>33</v>
       </c>
       <c r="X57" s="5" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="58" spans="1:24" x14ac:dyDescent="0.25">
@@ -8697,10 +8703,10 @@
         <v>34</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E58" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F58" s="6"/>
       <c r="G58" s="40" t="str">
@@ -8761,10 +8767,10 @@
         <v>35</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E59" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="40" t="str">
@@ -8781,7 +8787,7 @@
         <v>370</v>
       </c>
       <c r="M59" s="16" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="N59" s="16" t="s">
         <v>370</v>
@@ -8812,7 +8818,7 @@
         <v>35</v>
       </c>
       <c r="X59" s="5" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="60" spans="1:24" x14ac:dyDescent="0.25">
@@ -8827,10 +8833,10 @@
         <v>36</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E60" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F60" s="6"/>
       <c r="G60" s="40" t="str">
@@ -8891,10 +8897,10 @@
         <v>37</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E61" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F61" s="6"/>
       <c r="G61" s="40" t="str">
@@ -8911,10 +8917,10 @@
         <v>372</v>
       </c>
       <c r="M61" s="16" t="s">
-        <v>1361</v>
+        <v>1359</v>
       </c>
       <c r="N61" s="16" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
       <c r="O61" s="59" t="s">
         <v>412</v>
@@ -8955,10 +8961,10 @@
         <v>38</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E62" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="40" t="str">
@@ -8975,10 +8981,10 @@
         <v>373</v>
       </c>
       <c r="M62" s="16" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="N62" s="16" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="O62" s="59" t="s">
         <v>413</v>
@@ -9019,10 +9025,10 @@
         <v>39</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E63" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F63" s="6"/>
       <c r="G63" s="40" t="s">
@@ -9081,10 +9087,10 @@
         <v>40</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E64" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F64" s="6"/>
       <c r="G64" s="40" t="str">
@@ -9139,10 +9145,10 @@
         <v>41</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E65" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F65" s="6"/>
       <c r="G65" s="40" t="str">
@@ -9197,10 +9203,10 @@
         <v>42</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E66" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="40" t="str">
@@ -9255,10 +9261,10 @@
         <v>43</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E67" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="40" t="str">
@@ -9267,16 +9273,16 @@
       </c>
       <c r="H67" s="40"/>
       <c r="I67" s="5" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="J67" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K67" s="5" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="L67" s="19" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="M67" s="19"/>
       <c r="N67" s="19"/>
@@ -9319,7 +9325,7 @@
         <v>44</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E68" s="26"/>
       <c r="F68" s="6"/>
@@ -9374,7 +9380,7 @@
         <v>45</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E69" s="26">
         <v>99</v>
@@ -9391,7 +9397,7 @@
         <v>420</v>
       </c>
       <c r="L69" s="16" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="O69" s="59" t="s">
         <v>420</v>
@@ -9432,7 +9438,7 @@
         <v>46</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E70" s="26">
         <v>99</v>
@@ -9490,7 +9496,7 @@
         <v>47</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E71" s="26">
         <v>99</v>
@@ -9544,7 +9550,7 @@
         <v>48</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E72" s="26">
         <v>99</v>
@@ -9602,7 +9608,7 @@
         <v>697</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E73" s="26">
         <v>99</v>
@@ -9682,7 +9688,7 @@
       </c>
       <c r="Q74" s="59"/>
       <c r="R74" s="86" t="s">
-        <v>1395</v>
+        <v>1393</v>
       </c>
       <c r="S74" s="83" t="s">
         <v>557</v>
@@ -9708,10 +9714,10 @@
       </c>
       <c r="B75" s="2"/>
       <c r="C75" s="35" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="D75" s="25" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E75" s="26"/>
       <c r="F75" s="6"/>
@@ -9732,10 +9738,10 @@
       <c r="R75" s="83"/>
       <c r="S75" s="83"/>
       <c r="T75" s="20" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="V75" s="45" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="X75" s="2"/>
     </row>
@@ -9751,7 +9757,7 @@
         <v>51</v>
       </c>
       <c r="D76" s="25" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E76" s="26"/>
       <c r="F76" s="6"/>
@@ -9784,7 +9790,7 @@
         <v>558</v>
       </c>
       <c r="T76" s="2" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="U76" s="20" t="s">
         <v>51</v>
@@ -9809,10 +9815,10 @@
         <v>52</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E77" s="26" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F77" s="6"/>
       <c r="G77" s="40" t="str">
@@ -9826,10 +9832,10 @@
       <c r="I77" s="5"/>
       <c r="J77" s="5"/>
       <c r="K77" s="5" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="L77" s="49" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="M77" s="49"/>
       <c r="N77" s="49"/>
@@ -9868,10 +9874,10 @@
         <v>698</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E78" s="26" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F78" s="6"/>
       <c r="G78" s="40" t="str">
@@ -9880,16 +9886,16 @@
       </c>
       <c r="H78" s="40"/>
       <c r="I78" s="18" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="J78" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K78" s="5" t="s">
+        <v>1264</v>
+      </c>
+      <c r="L78" s="19" t="s">
         <v>1265</v>
-      </c>
-      <c r="L78" s="19" t="s">
-        <v>1266</v>
       </c>
       <c r="M78" s="19"/>
       <c r="N78" s="19"/>
@@ -9932,10 +9938,10 @@
         <v>699</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E79" s="26" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F79" s="6"/>
       <c r="G79" s="40" t="str">
@@ -9944,16 +9950,16 @@
       </c>
       <c r="H79" s="40"/>
       <c r="I79" s="19" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="J79" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K79" s="5" t="s">
+        <v>1165</v>
+      </c>
+      <c r="L79" s="49" t="s">
         <v>1166</v>
-      </c>
-      <c r="L79" s="49" t="s">
-        <v>1167</v>
       </c>
       <c r="M79" s="49"/>
       <c r="N79" s="49"/>
@@ -9996,10 +10002,10 @@
         <v>700</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E80" s="26" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F80" s="6"/>
       <c r="G80" s="40" t="str">
@@ -10056,10 +10062,10 @@
         <v>53</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E81" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F81" s="6"/>
       <c r="G81" s="40" t="str">
@@ -10071,16 +10077,16 @@
         <v>B02</v>
       </c>
       <c r="I81" s="18" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="J81" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K81" s="5" t="s">
+        <v>1167</v>
+      </c>
+      <c r="L81" s="49" t="s">
         <v>1168</v>
-      </c>
-      <c r="L81" s="49" t="s">
-        <v>1169</v>
       </c>
       <c r="M81" s="49"/>
       <c r="N81" s="49"/>
@@ -10123,10 +10129,10 @@
         <v>54</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E82" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F82" s="6"/>
       <c r="G82" s="40" t="str">
@@ -10138,16 +10144,16 @@
         <v>B03</v>
       </c>
       <c r="I82" s="18" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="J82" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K82" s="5" t="s">
+        <v>1169</v>
+      </c>
+      <c r="L82" s="49" t="s">
         <v>1170</v>
-      </c>
-      <c r="L82" s="49" t="s">
-        <v>1171</v>
       </c>
       <c r="M82" s="49"/>
       <c r="N82" s="49"/>
@@ -10192,10 +10198,10 @@
         <v>55</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F83" s="6"/>
       <c r="G83" s="40" t="str">
@@ -10207,16 +10213,16 @@
         <v>B04</v>
       </c>
       <c r="I83" s="16" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="J83" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K83" s="5" t="s">
+        <v>1238</v>
+      </c>
+      <c r="L83" s="49" t="s">
         <v>1239</v>
-      </c>
-      <c r="L83" s="49" t="s">
-        <v>1240</v>
       </c>
       <c r="M83" s="49"/>
       <c r="N83" s="49"/>
@@ -10259,10 +10265,10 @@
         <v>56</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="F84" s="6"/>
       <c r="G84" s="40" t="str">
@@ -10274,16 +10280,16 @@
         <v>B05</v>
       </c>
       <c r="I84" s="18" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="J84" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K84" s="5" t="s">
+        <v>1171</v>
+      </c>
+      <c r="L84" s="49" t="s">
         <v>1172</v>
-      </c>
-      <c r="L84" s="49" t="s">
-        <v>1173</v>
       </c>
       <c r="M84" s="49"/>
       <c r="N84" s="49"/>
@@ -10326,10 +10332,10 @@
         <v>57</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E85" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F85" s="6"/>
       <c r="G85" s="40" t="str">
@@ -10341,16 +10347,16 @@
         <v>B06</v>
       </c>
       <c r="I85" s="18" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="J85" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K85" s="5" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L85" s="49" t="s">
         <v>1174</v>
-      </c>
-      <c r="L85" s="49" t="s">
-        <v>1175</v>
       </c>
       <c r="M85" s="49"/>
       <c r="N85" s="49"/>
@@ -10393,10 +10399,10 @@
         <v>58</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E86" s="26" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="F86" s="6"/>
       <c r="G86" s="40" t="str">
@@ -10408,16 +10414,16 @@
         <v>B07</v>
       </c>
       <c r="I86" s="18" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="J86" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K86" s="5" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="L86" s="49" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="M86" s="49"/>
       <c r="N86" s="49"/>
@@ -10460,10 +10466,10 @@
         <v>59</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E87" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F87" s="6"/>
       <c r="G87" s="40" t="s">
@@ -10474,7 +10480,7 @@
         <v>B08</v>
       </c>
       <c r="J87" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K87" s="5" t="s">
         <v>952</v>
@@ -10519,10 +10525,10 @@
         <v>701</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E88" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F88" s="6"/>
       <c r="G88" s="40" t="str">
@@ -10531,16 +10537,16 @@
       </c>
       <c r="H88" s="40"/>
       <c r="I88" s="18" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="J88" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K88" s="5" t="s">
+        <v>1242</v>
+      </c>
+      <c r="L88" s="49" t="s">
         <v>1243</v>
-      </c>
-      <c r="L88" s="49" t="s">
-        <v>1244</v>
       </c>
       <c r="M88" s="49"/>
       <c r="N88" s="49"/>
@@ -10583,10 +10589,10 @@
         <v>702</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E89" s="26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F89" s="6"/>
       <c r="G89" s="40" t="str">
@@ -10595,16 +10601,16 @@
       </c>
       <c r="H89" s="40"/>
       <c r="I89" s="18" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="J89" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K89" s="5" t="s">
+        <v>1244</v>
+      </c>
+      <c r="L89" s="49" t="s">
         <v>1245</v>
-      </c>
-      <c r="L89" s="49" t="s">
-        <v>1246</v>
       </c>
       <c r="M89" s="49"/>
       <c r="N89" s="49"/>
@@ -10647,10 +10653,10 @@
         <v>60</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E90" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F90" s="6"/>
       <c r="G90" s="40" t="str">
@@ -10662,16 +10668,16 @@
         <v>B09</v>
       </c>
       <c r="I90" s="16" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="J90" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K90" s="5" t="s">
+        <v>1177</v>
+      </c>
+      <c r="L90" s="49" t="s">
         <v>1178</v>
-      </c>
-      <c r="L90" s="49" t="s">
-        <v>1179</v>
       </c>
       <c r="M90" s="49"/>
       <c r="N90" s="49"/>
@@ -10709,10 +10715,10 @@
       </c>
       <c r="B91" s="2"/>
       <c r="C91" s="37" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E91" s="26">
         <v>10</v>
@@ -10724,7 +10730,7 @@
         <v>B10</v>
       </c>
       <c r="J91" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K91" s="5"/>
       <c r="L91" s="49"/>
@@ -10736,11 +10742,11 @@
       <c r="R91" s="83"/>
       <c r="S91" s="83"/>
       <c r="T91" s="5" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="U91" s="20"/>
       <c r="V91" s="5" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="W91" s="45"/>
       <c r="X91" s="2"/>
@@ -10757,10 +10763,10 @@
         <v>61</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E92" s="26" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="F92" s="6"/>
       <c r="G92" s="40" t="str">
@@ -10769,16 +10775,16 @@
       </c>
       <c r="H92" s="40"/>
       <c r="I92" s="5" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="J92" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K92" s="5" t="s">
+        <v>1179</v>
+      </c>
+      <c r="L92" s="49" t="s">
         <v>1180</v>
-      </c>
-      <c r="L92" s="49" t="s">
-        <v>1181</v>
       </c>
       <c r="M92" s="49"/>
       <c r="N92" s="49"/>
@@ -10821,7 +10827,7 @@
         <v>62</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E93" s="26">
         <v>10</v>
@@ -10833,16 +10839,16 @@
       </c>
       <c r="H93" s="40"/>
       <c r="I93" s="5" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="J93" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K93" s="5" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="L93" s="49" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="M93" s="49"/>
       <c r="N93" s="49"/>
@@ -10885,7 +10891,7 @@
         <v>63</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E94" s="26">
         <v>11</v>
@@ -10900,16 +10906,16 @@
         <v>B11</v>
       </c>
       <c r="I94" s="5" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="J94" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K94" s="5" t="s">
+        <v>1205</v>
+      </c>
+      <c r="L94" s="49" t="s">
         <v>1206</v>
-      </c>
-      <c r="L94" s="49" t="s">
-        <v>1207</v>
       </c>
       <c r="M94" s="49"/>
       <c r="N94" s="49"/>
@@ -10952,10 +10958,10 @@
         <v>64</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E95" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F95" s="6"/>
       <c r="G95" s="40" t="str">
@@ -10967,16 +10973,16 @@
         <v>B12</v>
       </c>
       <c r="I95" s="19" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="J95" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K95" s="5" t="s">
+        <v>1181</v>
+      </c>
+      <c r="L95" s="49" t="s">
         <v>1182</v>
-      </c>
-      <c r="L95" s="49" t="s">
-        <v>1183</v>
       </c>
       <c r="M95" s="49"/>
       <c r="N95" s="49"/>
@@ -11019,7 +11025,7 @@
         <v>703</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E96" s="26">
         <v>99</v>
@@ -11031,16 +11037,16 @@
       </c>
       <c r="H96" s="40"/>
       <c r="I96" s="19" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="J96" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K96" s="5" t="s">
+        <v>1183</v>
+      </c>
+      <c r="L96" s="49" t="s">
         <v>1184</v>
-      </c>
-      <c r="L96" s="49" t="s">
-        <v>1185</v>
       </c>
       <c r="M96" s="49"/>
       <c r="N96" s="49"/>
@@ -11083,7 +11089,7 @@
         <v>704</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E97" s="26">
         <v>13</v>
@@ -11098,16 +11104,16 @@
         <v>B13</v>
       </c>
       <c r="I97" s="19" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="J97" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K97" s="5" t="s">
+        <v>1207</v>
+      </c>
+      <c r="L97" s="49" t="s">
         <v>1208</v>
-      </c>
-      <c r="L97" s="49" t="s">
-        <v>1209</v>
       </c>
       <c r="M97" s="49"/>
       <c r="N97" s="49"/>
@@ -11150,7 +11156,7 @@
         <v>705</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E98" s="26">
         <v>14</v>
@@ -11165,16 +11171,16 @@
         <v>B14</v>
       </c>
       <c r="I98" s="5" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="J98" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K98" s="5" t="s">
+        <v>1247</v>
+      </c>
+      <c r="L98" s="49" t="s">
         <v>1248</v>
-      </c>
-      <c r="L98" s="49" t="s">
-        <v>1249</v>
       </c>
       <c r="M98" s="49"/>
       <c r="N98" s="49"/>
@@ -11217,7 +11223,7 @@
         <v>706</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E99" s="26">
         <v>15</v>
@@ -11232,16 +11238,16 @@
         <v>B15</v>
       </c>
       <c r="I99" s="16" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="J99" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K99" s="5" t="s">
+        <v>1185</v>
+      </c>
+      <c r="L99" s="19" t="s">
         <v>1186</v>
-      </c>
-      <c r="L99" s="19" t="s">
-        <v>1187</v>
       </c>
       <c r="M99" s="19"/>
       <c r="N99" s="19"/>
@@ -11284,7 +11290,7 @@
         <v>707</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E100" s="26">
         <v>99</v>
@@ -11296,16 +11302,16 @@
       </c>
       <c r="H100" s="40"/>
       <c r="I100" s="19" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="J100" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K100" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="L100" s="49" t="s">
         <v>1188</v>
-      </c>
-      <c r="L100" s="49" t="s">
-        <v>1189</v>
       </c>
       <c r="M100" s="49"/>
       <c r="N100" s="49"/>
@@ -11348,7 +11354,7 @@
         <v>708</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E101" s="26">
         <v>99</v>
@@ -11360,16 +11366,16 @@
       </c>
       <c r="H101" s="40"/>
       <c r="I101" s="19" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="J101" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K101" s="5" t="s">
+        <v>1189</v>
+      </c>
+      <c r="L101" s="49" t="s">
         <v>1190</v>
-      </c>
-      <c r="L101" s="49" t="s">
-        <v>1191</v>
       </c>
       <c r="M101" s="49"/>
       <c r="N101" s="49"/>
@@ -11412,7 +11418,7 @@
         <v>709</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E102" s="26">
         <v>99</v>
@@ -11424,16 +11430,16 @@
       </c>
       <c r="H102" s="40"/>
       <c r="I102" s="19" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="J102" s="17" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K102" s="5" t="s">
+        <v>1191</v>
+      </c>
+      <c r="L102" s="49" t="s">
         <v>1192</v>
-      </c>
-      <c r="L102" s="49" t="s">
-        <v>1193</v>
       </c>
       <c r="M102" s="49"/>
       <c r="N102" s="49"/>
@@ -11476,7 +11482,7 @@
         <v>710</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E103" s="26">
         <v>99</v>
@@ -11536,7 +11542,7 @@
         <v>711</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E104" s="26">
         <v>16</v>
@@ -11596,7 +11602,7 @@
         <v>712</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E105" s="26">
         <v>16</v>
@@ -11661,7 +11667,7 @@
         <v>713</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E106" s="26">
         <v>16</v>
@@ -11726,13 +11732,13 @@
         <v>714</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E107" s="26">
         <v>16</v>
       </c>
       <c r="F107" s="6" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="G107" s="40" t="str">
         <f t="shared" si="10"/>
@@ -11791,7 +11797,7 @@
         <v>715</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E108" s="26">
         <v>17</v>
@@ -11854,7 +11860,7 @@
         <v>716</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="E109" s="26">
         <v>99</v>
@@ -11869,16 +11875,16 @@
         <v>B99</v>
       </c>
       <c r="I109" s="5" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="J109" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K109" s="5" t="s">
+        <v>1209</v>
+      </c>
+      <c r="L109" s="49" t="s">
         <v>1210</v>
-      </c>
-      <c r="L109" s="49" t="s">
-        <v>1211</v>
       </c>
       <c r="M109" s="49"/>
       <c r="N109" s="49"/>
@@ -11917,7 +11923,7 @@
         <v>65</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E110" s="26">
         <v>99</v>
@@ -11929,10 +11935,10 @@
       </c>
       <c r="H110" s="40"/>
       <c r="K110" s="5" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="L110" s="5" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="M110" s="5"/>
       <c r="N110" s="5"/>
@@ -11975,10 +11981,10 @@
         <v>66</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E111" s="26" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F111" s="6"/>
       <c r="G111" s="40" t="str">
@@ -11990,22 +11996,22 @@
         <v>D01</v>
       </c>
       <c r="I111" s="5" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="J111" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K111" s="5" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="L111" s="49" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="M111" s="49" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
       <c r="N111" s="49" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="O111" s="59" t="s">
         <v>975</v>
@@ -12033,7 +12039,7 @@
         <v>66</v>
       </c>
       <c r="X111" s="2" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="112" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
@@ -12048,10 +12054,10 @@
         <v>67</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E112" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F112" s="6"/>
       <c r="G112" s="40" t="s">
@@ -12064,18 +12070,18 @@
       <c r="I112" s="5"/>
       <c r="J112" s="5"/>
       <c r="K112" s="5" t="s">
+        <v>1304</v>
+      </c>
+      <c r="L112" s="19" t="s">
         <v>1305</v>
-      </c>
-      <c r="L112" s="19" t="s">
-        <v>1306</v>
       </c>
       <c r="M112" s="19"/>
       <c r="N112" s="19"/>
       <c r="O112" s="59" t="s">
+        <v>1304</v>
+      </c>
+      <c r="P112" s="62" t="s">
         <v>1305</v>
-      </c>
-      <c r="P112" s="62" t="s">
-        <v>1306</v>
       </c>
       <c r="Q112" s="65"/>
       <c r="R112" s="83" t="s">
@@ -12110,10 +12116,10 @@
         <v>717</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E113" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F113" s="6"/>
       <c r="G113" s="40" t="str">
@@ -12170,10 +12176,10 @@
         <v>718</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E114" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F114" s="6"/>
       <c r="G114" s="40" t="str">
@@ -12230,10 +12236,10 @@
         <v>719</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E115" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F115" s="6"/>
       <c r="G115" s="40" t="str">
@@ -12290,10 +12296,10 @@
         <v>720</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E116" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F116" s="6"/>
       <c r="G116" s="40" t="str">
@@ -12404,13 +12410,13 @@
       </c>
       <c r="B118" s="2"/>
       <c r="C118" s="32" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E118" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F118" s="6"/>
       <c r="G118" s="40" t="s">
@@ -12432,11 +12438,11 @@
       <c r="R118" s="83"/>
       <c r="S118" s="83"/>
       <c r="T118" s="2" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="U118" s="20"/>
       <c r="V118" s="2" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
       <c r="W118" s="45"/>
       <c r="X118" s="2"/>
@@ -12448,13 +12454,13 @@
       </c>
       <c r="B119" s="2"/>
       <c r="C119" s="32" t="s">
-        <v>1392</v>
+        <v>1390</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E119" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F119" s="6"/>
       <c r="G119" s="40"/>
@@ -12474,11 +12480,11 @@
       <c r="R119" s="83"/>
       <c r="S119" s="83"/>
       <c r="T119" s="2" t="s">
-        <v>1393</v>
+        <v>1391</v>
       </c>
       <c r="U119" s="20"/>
       <c r="V119" s="2" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="W119" s="45"/>
       <c r="X119" s="2"/>
@@ -12490,7 +12496,7 @@
       </c>
       <c r="B120" s="2"/>
       <c r="C120" s="35" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="D120" s="6"/>
       <c r="E120" s="26"/>
@@ -12575,10 +12581,10 @@
         <v>723</v>
       </c>
       <c r="D122" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E122" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F122" s="6"/>
       <c r="G122" s="40" t="str">
@@ -12635,10 +12641,10 @@
         <v>724</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E123" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F123" s="6"/>
       <c r="G123" s="40" t="str">
@@ -12695,10 +12701,10 @@
         <v>725</v>
       </c>
       <c r="D124" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E124" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F124" s="6"/>
       <c r="G124" s="40" t="str">
@@ -12755,10 +12761,10 @@
         <v>69</v>
       </c>
       <c r="D125" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E125" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F125" s="6"/>
       <c r="G125" s="40" t="str">
@@ -12772,13 +12778,13 @@
         <v>443</v>
       </c>
       <c r="L125" s="49" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="M125" s="49" t="s">
         <v>443</v>
       </c>
       <c r="N125" s="49" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="O125" s="59" t="s">
         <v>443</v>
@@ -12819,10 +12825,10 @@
         <v>70</v>
       </c>
       <c r="D126" s="27" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E126" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F126" s="6" t="s">
         <v>1126</v>
@@ -12836,24 +12842,24 @@
         <v>D04a</v>
       </c>
       <c r="I126" s="5" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="J126" s="5" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="K126" s="5" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
       <c r="L126" s="19" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="M126" s="19"/>
       <c r="N126" s="19"/>
       <c r="O126" s="59" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="P126" s="62" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="Q126" s="65"/>
       <c r="R126" s="83" t="s">
@@ -12941,10 +12947,10 @@
         <v>668</v>
       </c>
       <c r="D128" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E128" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>1127</v>
@@ -12958,14 +12964,14 @@
         <v>D04b</v>
       </c>
       <c r="I128" s="79" t="s">
-        <v>1387</v>
+        <v>1385</v>
       </c>
       <c r="J128" s="5"/>
       <c r="K128" s="5" t="s">
-        <v>1382</v>
+        <v>1380</v>
       </c>
       <c r="L128" s="49" t="s">
-        <v>1382</v>
+        <v>1380</v>
       </c>
       <c r="M128" s="49"/>
       <c r="N128" s="49"/>
@@ -13008,13 +13014,13 @@
         <v>669</v>
       </c>
       <c r="D129" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E129" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F129" s="28" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="G129" s="40" t="str">
         <f t="shared" si="11"/>
@@ -13073,13 +13079,13 @@
         <v>726</v>
       </c>
       <c r="D130" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E130" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F130" s="28" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="G130" s="40" t="str">
         <f t="shared" si="11"/>
@@ -13138,10 +13144,10 @@
         <v>727</v>
       </c>
       <c r="D131" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E131" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F131" s="6"/>
       <c r="G131" s="40" t="str">
@@ -13193,10 +13199,10 @@
         <v>728</v>
       </c>
       <c r="D132" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E132" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F132" s="6"/>
       <c r="G132" s="40" t="str">
@@ -13205,16 +13211,16 @@
       </c>
       <c r="H132" s="40"/>
       <c r="I132" s="79" t="s">
-        <v>1401</v>
+        <v>1399</v>
       </c>
       <c r="J132" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K132" s="5" t="s">
-        <v>1388</v>
+        <v>1386</v>
       </c>
       <c r="L132" s="19" t="s">
-        <v>1389</v>
+        <v>1387</v>
       </c>
       <c r="M132" s="19"/>
       <c r="N132" s="19"/>
@@ -13244,7 +13250,7 @@
         <v>728</v>
       </c>
       <c r="X132" s="2" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="133" spans="1:24" x14ac:dyDescent="0.25">
@@ -13259,10 +13265,10 @@
         <v>72</v>
       </c>
       <c r="D133" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E133" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F133" s="6"/>
       <c r="G133" s="40" t="str">
@@ -13315,10 +13321,10 @@
         <v>73</v>
       </c>
       <c r="D134" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E134" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F134" s="6"/>
       <c r="G134" s="40" t="str">
@@ -13375,10 +13381,10 @@
         <v>729</v>
       </c>
       <c r="D135" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E135" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F135" s="6"/>
       <c r="G135" s="40" t="str">
@@ -13480,10 +13486,10 @@
         <v>730</v>
       </c>
       <c r="D137" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E137" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F137" s="6"/>
       <c r="G137" s="40" t="str">
@@ -13536,10 +13542,10 @@
         <v>731</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E138" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F138" s="6"/>
       <c r="G138" s="40" t="str">
@@ -13592,10 +13598,10 @@
         <v>75</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E139" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F139" s="6"/>
       <c r="G139" s="40" t="str">
@@ -13648,10 +13654,10 @@
         <v>76</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E140" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F140" s="6"/>
       <c r="G140" s="40" t="str">
@@ -13763,10 +13769,10 @@
         <v>732</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E142" s="26" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="F142" s="6"/>
       <c r="G142" s="40" t="str">
@@ -13826,10 +13832,10 @@
         <v>79</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E143" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F143" s="6"/>
       <c r="G143" s="40" t="str">
@@ -13886,10 +13892,10 @@
         <v>80</v>
       </c>
       <c r="D144" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E144" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F144" s="6"/>
       <c r="G144" s="40" t="str">
@@ -13946,10 +13952,10 @@
         <v>81</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E145" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F145" s="6"/>
       <c r="G145" s="40" t="str">
@@ -14006,10 +14012,10 @@
         <v>82</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E146" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F146" s="6"/>
       <c r="G146" s="40" t="str">
@@ -14062,10 +14068,10 @@
         <v>83</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E147" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F147" s="6"/>
       <c r="G147" s="40" t="str">
@@ -14118,10 +14124,10 @@
         <v>84</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E148" s="26" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="F148" s="6"/>
       <c r="G148" s="40" t="str">
@@ -14133,16 +14139,16 @@
         <v>D06</v>
       </c>
       <c r="I148" s="57" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="J148" s="18" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K148" s="5" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="L148" s="58" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="M148" s="58"/>
       <c r="N148" s="58"/>
@@ -14240,7 +14246,7 @@
         <v>86</v>
       </c>
       <c r="D150" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E150" s="26">
         <v>99</v>
@@ -14296,7 +14302,7 @@
         <v>87</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E151" s="26">
         <v>99</v>
@@ -14352,7 +14358,7 @@
         <v>733</v>
       </c>
       <c r="D152" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E152" s="26">
         <v>99</v>
@@ -14408,7 +14414,7 @@
         <v>89</v>
       </c>
       <c r="D153" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E153" s="26">
         <v>99</v>
@@ -14464,7 +14470,7 @@
         <v>90</v>
       </c>
       <c r="D154" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E154" s="26">
         <v>99</v>
@@ -14481,7 +14487,7 @@
         <v>460</v>
       </c>
       <c r="L154" s="49" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="M154" s="49"/>
       <c r="N154" s="49"/>
@@ -14520,7 +14526,7 @@
         <v>91</v>
       </c>
       <c r="D155" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E155" s="26">
         <v>99</v>
@@ -14576,7 +14582,7 @@
         <v>92</v>
       </c>
       <c r="D156" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E156" s="26">
         <v>99</v>
@@ -14634,7 +14640,7 @@
         <v>93</v>
       </c>
       <c r="D157" s="25" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E157" s="26"/>
       <c r="F157" s="6"/>
@@ -14692,7 +14698,7 @@
         <v>94</v>
       </c>
       <c r="D158" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E158" s="26">
         <v>99</v>
@@ -14715,7 +14721,7 @@
         <v>464</v>
       </c>
       <c r="N158" s="49" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
       <c r="O158" s="59" t="s">
         <v>464</v>
@@ -14756,10 +14762,10 @@
         <v>95</v>
       </c>
       <c r="D159" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E159" s="26" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F159" s="6"/>
       <c r="G159" s="40" t="str">
@@ -14823,10 +14829,10 @@
         <v>96</v>
       </c>
       <c r="D160" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E160" s="26" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="F160" s="6"/>
       <c r="G160" s="40" t="str">
@@ -14890,10 +14896,10 @@
         <v>97</v>
       </c>
       <c r="D161" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E161" s="26" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="F161" s="6"/>
       <c r="G161" s="40" t="str">
@@ -14905,22 +14911,22 @@
         <v>C03</v>
       </c>
       <c r="I161" s="5" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="J161" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K161" s="5" t="s">
+        <v>1225</v>
+      </c>
+      <c r="L161" s="49" t="s">
         <v>1226</v>
       </c>
-      <c r="L161" s="49" t="s">
-        <v>1227</v>
-      </c>
       <c r="M161" s="49" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="N161" s="49" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="O161" s="59" t="s">
         <v>467</v>
@@ -14961,10 +14967,10 @@
         <v>98</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E162" s="26" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="F162" s="6"/>
       <c r="G162" s="40" t="str">
@@ -14984,10 +14990,10 @@
         <v>830</v>
       </c>
       <c r="M162" s="49" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
       <c r="N162" s="49" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="O162" s="59" t="s">
         <v>468</v>
@@ -15015,7 +15021,7 @@
         <v>98</v>
       </c>
       <c r="X162" s="76" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="163" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
@@ -15026,10 +15032,10 @@
       <c r="B163" s="2"/>
       <c r="C163" s="36"/>
       <c r="D163" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E163" s="26" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="F163" s="6"/>
       <c r="G163" s="40" t="str">
@@ -15041,22 +15047,22 @@
         <v>C05</v>
       </c>
       <c r="I163" s="5" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="J163" s="5" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="K163" s="5" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="L163" s="49" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="M163" s="49" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="N163" s="49" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="O163" s="59"/>
       <c r="P163" s="64"/>
@@ -15064,7 +15070,7 @@
       <c r="R163" s="83"/>
       <c r="S163" s="83"/>
       <c r="T163" s="5" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="U163" s="50"/>
       <c r="V163" s="5"/>
@@ -15083,7 +15089,7 @@
         <v>99</v>
       </c>
       <c r="D164" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="E164" s="26">
         <v>99</v>
@@ -15098,22 +15104,22 @@
         <v>C99</v>
       </c>
       <c r="I164" s="5" t="s">
+        <v>1321</v>
+      </c>
+      <c r="J164" s="5" t="s">
         <v>1322</v>
       </c>
-      <c r="J164" s="5" t="s">
+      <c r="K164" s="5" t="s">
         <v>1323</v>
       </c>
-      <c r="K164" s="5" t="s">
+      <c r="L164" s="19" t="s">
         <v>1324</v>
       </c>
-      <c r="L164" s="19" t="s">
-        <v>1325</v>
-      </c>
       <c r="M164" s="19" t="s">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="N164" s="19" t="s">
-        <v>1345</v>
+        <v>1343</v>
       </c>
       <c r="O164" s="59" t="s">
         <v>469</v>
@@ -15129,7 +15135,7 @@
         <v>1102</v>
       </c>
       <c r="T164" s="74" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="U164" s="52" t="s">
         <v>99</v>
@@ -15141,7 +15147,7 @@
         <v>99</v>
       </c>
       <c r="X164" s="76" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="165" spans="1:24" x14ac:dyDescent="0.25">
@@ -15213,10 +15219,10 @@
         <v>101</v>
       </c>
       <c r="D166" s="27" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E166" s="78" t="s">
-        <v>1351</v>
+        <v>1349</v>
       </c>
       <c r="F166" s="6"/>
       <c r="G166" s="40" t="str">
@@ -15276,10 +15282,10 @@
         <v>102</v>
       </c>
       <c r="D167" s="27" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E167" s="78" t="s">
-        <v>1352</v>
+        <v>1350</v>
       </c>
       <c r="F167" s="6"/>
       <c r="G167" s="40" t="str">
@@ -15336,13 +15342,13 @@
         <v>157</v>
       </c>
       <c r="C168" s="31" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="D168" s="27" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E168" s="78" t="s">
-        <v>1353</v>
+        <v>1351</v>
       </c>
       <c r="F168" s="6"/>
       <c r="G168" s="40" t="str">
@@ -15402,10 +15408,10 @@
         <v>104</v>
       </c>
       <c r="D169" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E169" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F169" s="6"/>
       <c r="G169" s="40" t="s">
@@ -15439,10 +15445,10 @@
         <v>682</v>
       </c>
       <c r="T169" s="76" t="s">
+        <v>1328</v>
+      </c>
+      <c r="U169" s="20" t="s">
         <v>1329</v>
-      </c>
-      <c r="U169" s="20" t="s">
-        <v>1330</v>
       </c>
       <c r="V169" s="2" t="s">
         <v>281</v>
@@ -15464,10 +15470,10 @@
         <v>105</v>
       </c>
       <c r="D170" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E170" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F170" s="6"/>
       <c r="G170" s="40" t="str">
@@ -15524,10 +15530,10 @@
         <v>106</v>
       </c>
       <c r="D171" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E171" s="26" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="F171" s="6"/>
       <c r="G171" s="40" t="str">
@@ -15539,16 +15545,16 @@
         <v>D11</v>
       </c>
       <c r="I171" s="16" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="J171" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K171" s="5" t="s">
+        <v>1200</v>
+      </c>
+      <c r="L171" s="49" t="s">
         <v>1201</v>
-      </c>
-      <c r="L171" s="49" t="s">
-        <v>1202</v>
       </c>
       <c r="M171" s="49"/>
       <c r="N171" s="49"/>
@@ -15591,10 +15597,10 @@
         <v>107</v>
       </c>
       <c r="D172" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E172" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F172" s="6"/>
       <c r="G172" s="40" t="str">
@@ -15651,10 +15657,10 @@
         <v>734</v>
       </c>
       <c r="D173" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E173" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F173" s="6"/>
       <c r="G173" s="40" t="str">
@@ -15711,10 +15717,10 @@
         <v>735</v>
       </c>
       <c r="D174" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E174" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F174" s="6"/>
       <c r="G174" s="40" t="str">
@@ -15771,10 +15777,10 @@
         <v>667</v>
       </c>
       <c r="D175" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E175" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F175" s="6"/>
       <c r="G175" s="40" t="str">
@@ -15831,10 +15837,10 @@
         <v>736</v>
       </c>
       <c r="D176" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E176" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F176" s="6"/>
       <c r="G176" s="40" t="str">
@@ -15891,10 +15897,10 @@
         <v>737</v>
       </c>
       <c r="D177" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E177" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F177" s="6"/>
       <c r="G177" s="40" t="str">
@@ -15951,10 +15957,10 @@
         <v>738</v>
       </c>
       <c r="D178" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E178" s="26" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="F178" s="6"/>
       <c r="G178" s="40" t="str">
@@ -15963,16 +15969,16 @@
       </c>
       <c r="H178" s="40"/>
       <c r="I178" s="5" t="s">
+        <v>1202</v>
+      </c>
+      <c r="J178" s="5" t="s">
+        <v>1159</v>
+      </c>
+      <c r="K178" s="5" t="s">
         <v>1203</v>
       </c>
-      <c r="J178" s="5" t="s">
-        <v>1160</v>
-      </c>
-      <c r="K178" s="5" t="s">
+      <c r="L178" s="49" t="s">
         <v>1204</v>
-      </c>
-      <c r="L178" s="49" t="s">
-        <v>1205</v>
       </c>
       <c r="M178" s="49"/>
       <c r="N178" s="49"/>
@@ -16070,10 +16076,10 @@
         <v>109</v>
       </c>
       <c r="D180" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E180" s="26" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="F180" s="6"/>
       <c r="G180" s="40" t="s">
@@ -16134,10 +16140,10 @@
         <v>739</v>
       </c>
       <c r="D181" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E181" s="26" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="F181" s="6" t="s">
         <v>1126</v>
@@ -16201,10 +16207,10 @@
         <v>740</v>
       </c>
       <c r="D182" s="27" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E182" s="26" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="F182" s="6" t="s">
         <v>1127</v>
@@ -16268,13 +16274,13 @@
         <v>741</v>
       </c>
       <c r="D183" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E183" s="26" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="F183" s="6" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="G183" s="40" t="str">
         <f t="shared" si="18"/>
@@ -16335,7 +16341,7 @@
         <v>742</v>
       </c>
       <c r="D184" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E184" s="26">
         <v>99</v>
@@ -16391,7 +16397,7 @@
         <v>110</v>
       </c>
       <c r="D185" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E185" s="26">
         <v>99</v>
@@ -16451,7 +16457,7 @@
         <v>743</v>
       </c>
       <c r="D186" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E186" s="26">
         <v>99</v>
@@ -16511,7 +16517,7 @@
         <v>112</v>
       </c>
       <c r="D187" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E187" s="26">
         <v>99</v>
@@ -16571,7 +16577,7 @@
         <v>113</v>
       </c>
       <c r="D188" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E188" s="26">
         <v>99</v>
@@ -16631,7 +16637,7 @@
         <v>114</v>
       </c>
       <c r="D189" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E189" s="26">
         <v>99</v>
@@ -16748,7 +16754,7 @@
         <v>116</v>
       </c>
       <c r="D191" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E191" s="26">
         <v>99</v>
@@ -16808,7 +16814,7 @@
         <v>117</v>
       </c>
       <c r="D192" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E192" s="26">
         <v>99</v>
@@ -16864,7 +16870,7 @@
         <v>118</v>
       </c>
       <c r="D193" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E193" s="26">
         <v>99</v>
@@ -16920,7 +16926,7 @@
         <v>119</v>
       </c>
       <c r="D194" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E194" s="26">
         <v>99</v>
@@ -16976,7 +16982,7 @@
         <v>120</v>
       </c>
       <c r="D195" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E195" s="26">
         <v>99</v>
@@ -16988,16 +16994,16 @@
       </c>
       <c r="H195" s="40"/>
       <c r="I195" s="5" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="J195" s="5" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="K195" s="5" t="s">
+        <v>1197</v>
+      </c>
+      <c r="L195" s="49" t="s">
         <v>1198</v>
-      </c>
-      <c r="L195" s="49" t="s">
-        <v>1199</v>
       </c>
       <c r="M195" s="49"/>
       <c r="N195" s="49"/>
@@ -17040,10 +17046,10 @@
         <v>121</v>
       </c>
       <c r="D196" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E196" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F196" s="6"/>
       <c r="G196" s="40" t="s">
@@ -17102,10 +17108,10 @@
         <v>122</v>
       </c>
       <c r="D197" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E197" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F197" s="6"/>
       <c r="G197" s="40" t="str">
@@ -17162,10 +17168,10 @@
         <v>123</v>
       </c>
       <c r="D198" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E198" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F198" s="6"/>
       <c r="G198" s="40" t="str">
@@ -17222,10 +17228,10 @@
         <v>124</v>
       </c>
       <c r="D199" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E199" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F199" s="6"/>
       <c r="G199" s="40" t="str">
@@ -17282,10 +17288,10 @@
         <v>125</v>
       </c>
       <c r="D200" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E200" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F200" s="6"/>
       <c r="G200" s="40" t="str">
@@ -17342,10 +17348,10 @@
         <v>126</v>
       </c>
       <c r="D201" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E201" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F201" s="6"/>
       <c r="G201" s="40" t="str">
@@ -17402,10 +17408,10 @@
         <v>127</v>
       </c>
       <c r="D202" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E202" s="26" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="F202" s="6"/>
       <c r="G202" s="40" t="str">
@@ -17515,7 +17521,7 @@
         <v>129</v>
       </c>
       <c r="D204" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E204" s="26">
         <v>99</v>
@@ -17571,7 +17577,7 @@
         <v>130</v>
       </c>
       <c r="D205" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E205" s="26">
         <v>99</v>
@@ -17627,7 +17633,7 @@
         <v>131</v>
       </c>
       <c r="D206" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E206" s="26">
         <v>99</v>
@@ -17683,7 +17689,7 @@
         <v>744</v>
       </c>
       <c r="D207" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E207" s="26">
         <v>99</v>
@@ -17739,7 +17745,7 @@
         <v>132</v>
       </c>
       <c r="D208" s="25" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E208" s="26"/>
       <c r="F208" s="6"/>
@@ -17766,7 +17772,7 @@
       </c>
       <c r="Q208" s="62"/>
       <c r="R208" s="86" t="s">
-        <v>1396</v>
+        <v>1394</v>
       </c>
       <c r="S208" s="83" t="s">
         <v>654</v>
@@ -17788,7 +17794,7 @@
     <row r="209" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A209" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>...E.01. - Unintentional injuries</v>
+        <v/>
       </c>
       <c r="B209" s="2">
         <v>198</v>
@@ -17797,17 +17803,14 @@
         <v>133</v>
       </c>
       <c r="D209" s="6" t="s">
-        <v>1142</v>
+        <v>952</v>
       </c>
       <c r="E209" s="26" t="s">
-        <v>1143</v>
+        <v>952</v>
       </c>
       <c r="F209" s="6"/>
       <c r="G209" s="40"/>
-      <c r="H209" s="40" t="str">
-        <f>CONCATENATE(D209,E209,F209)</f>
-        <v>E01</v>
-      </c>
+      <c r="H209" s="40"/>
       <c r="I209" s="5"/>
       <c r="J209" s="5"/>
       <c r="K209" s="5" t="s">
@@ -17848,7 +17851,7 @@
     <row r="210" spans="1:24" ht="36" x14ac:dyDescent="0.25">
       <c r="A210" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.01.a. - Road injury</v>
+        <v>....E.01. . - Road injury</v>
       </c>
       <c r="B210" s="2">
         <v>199</v>
@@ -17857,33 +17860,33 @@
         <v>134</v>
       </c>
       <c r="D210" s="6" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E210" s="26" t="s">
         <v>1142</v>
       </c>
-      <c r="E210" s="26" t="s">
-        <v>1143</v>
-      </c>
-      <c r="F210" s="6" t="s">
-        <v>1126</v>
+      <c r="F210" s="88" t="s">
+        <v>952</v>
       </c>
       <c r="G210" s="40" t="str">
         <f t="shared" ref="G210:G219" si="21">CONCATENATE("c",D210,E210,F210)</f>
-        <v>cE01a</v>
+        <v xml:space="preserve">cE01 </v>
       </c>
       <c r="H210" s="40" t="str">
         <f>CONCATENATE(D210,E210,F210)</f>
-        <v>E01a</v>
+        <v xml:space="preserve">E01 </v>
       </c>
       <c r="I210" s="5" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="J210" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K210" s="5" t="s">
+        <v>1193</v>
+      </c>
+      <c r="L210" s="19" t="s">
         <v>1194</v>
-      </c>
-      <c r="L210" s="19" t="s">
-        <v>1195</v>
       </c>
       <c r="M210" s="19"/>
       <c r="N210" s="19"/>
@@ -17917,36 +17920,36 @@
     <row r="211" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A211" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.01.b. - Substance use-associated poisonings</v>
+        <v>....E.02. . - Substance use-associated poisonings</v>
       </c>
       <c r="B211" s="2"/>
       <c r="C211" s="31" t="s">
-        <v>1383</v>
+        <v>1381</v>
       </c>
       <c r="D211" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E211" s="26" t="s">
         <v>1143</v>
       </c>
-      <c r="F211" s="6" t="s">
-        <v>1127</v>
+      <c r="F211" s="88" t="s">
+        <v>952</v>
       </c>
       <c r="G211" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01b</v>
+        <v xml:space="preserve">cE02 </v>
       </c>
       <c r="H211" s="40" t="str">
         <f t="shared" ref="H211:H212" si="22">CONCATENATE(D211,E211,F211)</f>
-        <v>E01b</v>
+        <v xml:space="preserve">E02 </v>
       </c>
       <c r="I211" s="5"/>
       <c r="J211" s="5"/>
       <c r="K211" s="79" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
       <c r="L211" s="80" t="s">
-        <v>1385</v>
+        <v>1383</v>
       </c>
       <c r="M211" s="19"/>
       <c r="N211" s="19"/>
@@ -17956,7 +17959,7 @@
       <c r="R211" s="83"/>
       <c r="S211" s="83"/>
       <c r="T211" s="5" t="s">
-        <v>1394</v>
+        <v>1392</v>
       </c>
       <c r="U211" s="20"/>
       <c r="V211" s="5"/>
@@ -17966,38 +17969,38 @@
     <row r="212" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A212" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.01.c. - Poisonings (non-substance use)</v>
+        <v>....E.03. . - Poisonings (non-substance use)</v>
       </c>
       <c r="B212" s="2">
         <v>200</v>
       </c>
       <c r="C212" s="31" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="D212" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E212" s="26" t="s">
-        <v>1143</v>
-      </c>
-      <c r="F212" s="6" t="s">
-        <v>1130</v>
+        <v>1144</v>
+      </c>
+      <c r="F212" s="88" t="s">
+        <v>952</v>
       </c>
       <c r="G212" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01c</v>
+        <v xml:space="preserve">cE03 </v>
       </c>
       <c r="H212" s="40" t="str">
         <f t="shared" si="22"/>
-        <v>E01c</v>
+        <v xml:space="preserve">E03 </v>
       </c>
       <c r="I212" s="5"/>
       <c r="J212" s="5"/>
       <c r="K212" s="79" t="s">
-        <v>1391</v>
+        <v>1389</v>
       </c>
       <c r="L212" s="81" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
       <c r="M212" s="49"/>
       <c r="N212" s="49"/>
@@ -18015,7 +18018,7 @@
         <v>1006</v>
       </c>
       <c r="T212" s="5" t="s">
-        <v>1402</v>
+        <v>1400</v>
       </c>
       <c r="U212" s="20" t="s">
         <v>135</v>
@@ -18031,7 +18034,7 @@
     <row r="213" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A213" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.01.d. - Falls</v>
+        <v>....E.04. . - Falls</v>
       </c>
       <c r="B213" s="2">
         <v>201</v>
@@ -18040,21 +18043,21 @@
         <v>136</v>
       </c>
       <c r="D213" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E213" s="26" t="s">
-        <v>1143</v>
-      </c>
-      <c r="F213" s="6" t="s">
-        <v>1153</v>
+        <v>1145</v>
+      </c>
+      <c r="F213" s="88" t="s">
+        <v>952</v>
       </c>
       <c r="G213" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01d</v>
+        <v xml:space="preserve">cE04 </v>
       </c>
       <c r="H213" s="40" t="str">
         <f>CONCATENATE(D213,E213,F213)</f>
-        <v>E01d</v>
+        <v xml:space="preserve">E04 </v>
       </c>
       <c r="I213" s="5" t="s">
         <v>952</v>
@@ -18107,17 +18110,17 @@
         <v>137</v>
       </c>
       <c r="D214" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E214" s="26" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="F214" s="6" t="s">
-        <v>1128</v>
+        <v>952</v>
       </c>
       <c r="G214" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01x</v>
+        <v xml:space="preserve">cE05 </v>
       </c>
       <c r="H214" s="40"/>
       <c r="K214" s="5" t="s">
@@ -18167,17 +18170,17 @@
         <v>745</v>
       </c>
       <c r="D215" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E215" s="26" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="F215" s="6" t="s">
-        <v>1128</v>
+        <v>952</v>
       </c>
       <c r="G215" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01x</v>
+        <v xml:space="preserve">cE05 </v>
       </c>
       <c r="H215" s="40"/>
       <c r="I215" s="5"/>
@@ -18229,26 +18232,26 @@
         <v>746</v>
       </c>
       <c r="D216" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E216" s="26" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="F216" s="6" t="s">
-        <v>1128</v>
+        <v>952</v>
       </c>
       <c r="G216" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01x</v>
+        <v xml:space="preserve">cE05 </v>
       </c>
       <c r="H216" s="40"/>
       <c r="I216" s="5"/>
       <c r="J216" s="5"/>
       <c r="K216" s="5" t="s">
+        <v>1377</v>
+      </c>
+      <c r="L216" s="49" t="s">
         <v>1379</v>
-      </c>
-      <c r="L216" s="49" t="s">
-        <v>1381</v>
       </c>
       <c r="M216" s="49"/>
       <c r="N216" s="49"/>
@@ -18282,39 +18285,39 @@
     <row r="217" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A217" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.01.x. - Accidental Firearm</v>
+        <v>....E.05. . - Accidental Firearm</v>
       </c>
       <c r="B217" s="2"/>
       <c r="C217" s="31" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="D217" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E217" s="26" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="F217" s="6" t="s">
-        <v>1128</v>
+        <v>952</v>
       </c>
       <c r="G217" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01x</v>
+        <v xml:space="preserve">cE05 </v>
       </c>
       <c r="H217" s="40" t="s">
         <v>952</v>
       </c>
       <c r="I217" s="5" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="J217" s="5" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="K217" s="5" t="s">
-        <v>1375</v>
+        <v>1373</v>
       </c>
       <c r="L217" s="49" t="s">
-        <v>1376</v>
+        <v>1374</v>
       </c>
       <c r="M217" s="49"/>
       <c r="N217" s="49"/>
@@ -18324,7 +18327,7 @@
       <c r="R217" s="83"/>
       <c r="S217" s="83"/>
       <c r="T217" s="5" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="U217" s="20"/>
       <c r="V217" s="5"/>
@@ -18343,30 +18346,30 @@
         <v>747</v>
       </c>
       <c r="D218" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E218" s="26" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="F218" s="6" t="s">
-        <v>1128</v>
+        <v>952</v>
       </c>
       <c r="G218" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01x</v>
+        <v xml:space="preserve">cE05 </v>
       </c>
       <c r="H218" s="40"/>
       <c r="I218" s="5" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="J218" s="5" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K218" s="5" t="s">
+        <v>1195</v>
+      </c>
+      <c r="L218" s="49" t="s">
         <v>1196</v>
-      </c>
-      <c r="L218" s="49" t="s">
-        <v>1197</v>
       </c>
       <c r="M218" s="49"/>
       <c r="N218" s="49"/>
@@ -18396,7 +18399,7 @@
     <row r="219" spans="1:24" ht="33" x14ac:dyDescent="0.25">
       <c r="A219" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.01.x. - Other unintentional injuries</v>
+        <v>....E.05. . - Other unintentional injuries</v>
       </c>
       <c r="B219" s="2">
         <v>206</v>
@@ -18405,33 +18408,33 @@
         <v>748</v>
       </c>
       <c r="D219" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E219" s="26" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="F219" s="6" t="s">
-        <v>1128</v>
+        <v>952</v>
       </c>
       <c r="G219" s="40" t="str">
         <f t="shared" si="21"/>
-        <v>cE01x</v>
+        <v xml:space="preserve">cE05 </v>
       </c>
       <c r="H219" s="40" t="str">
         <f>CONCATENATE(D219,E219,F219)</f>
-        <v>E01x</v>
+        <v xml:space="preserve">E05 </v>
       </c>
       <c r="I219" s="5" t="s">
-        <v>1400</v>
+        <v>1398</v>
       </c>
       <c r="J219" s="5" t="s">
+        <v>1253</v>
+      </c>
+      <c r="K219" s="5" t="s">
         <v>1254</v>
       </c>
-      <c r="K219" s="5" t="s">
+      <c r="L219" s="49" t="s">
         <v>1255</v>
-      </c>
-      <c r="L219" s="49" t="s">
-        <v>1256</v>
       </c>
       <c r="M219" s="49"/>
       <c r="N219" s="49"/>
@@ -18461,7 +18464,7 @@
         <v>887</v>
       </c>
       <c r="X219" s="22" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="220" spans="1:24" ht="16.5" x14ac:dyDescent="0.25">
@@ -18520,7 +18523,7 @@
     <row r="221" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A221" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>...E.02. - Suicide/Self-harm</v>
+        <v>...E.07. - Suicide/Self-harm</v>
       </c>
       <c r="B221" s="2">
         <v>208</v>
@@ -18529,31 +18532,31 @@
         <v>140</v>
       </c>
       <c r="D221" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E221" s="26" t="s">
-        <v>1144</v>
+        <v>1148</v>
       </c>
       <c r="F221" s="6"/>
       <c r="G221" s="40" t="str">
         <f t="shared" ref="G221:G228" si="23">CONCATENATE("c",D221,E221,F221)</f>
-        <v>cE02</v>
+        <v>cE07</v>
       </c>
       <c r="H221" s="40" t="str">
         <f>CONCATENATE(D221,E221,F221)</f>
-        <v>E02</v>
+        <v>E07</v>
       </c>
       <c r="I221" s="5" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="J221" s="5" t="s">
+        <v>1211</v>
+      </c>
+      <c r="K221" s="5" t="s">
         <v>1212</v>
       </c>
-      <c r="K221" s="5" t="s">
+      <c r="L221" s="49" t="s">
         <v>1213</v>
-      </c>
-      <c r="L221" s="49" t="s">
-        <v>1214</v>
       </c>
       <c r="M221" s="49"/>
       <c r="N221" s="49"/>
@@ -18571,7 +18574,7 @@
         <v>999</v>
       </c>
       <c r="T221" s="5" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="U221" s="20" t="s">
         <v>140</v>
@@ -18587,7 +18590,7 @@
     <row r="222" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A222" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>...E.03. - Homicide/Interpersonal violence</v>
+        <v>...E.08. - Homicide/Interpersonal violence</v>
       </c>
       <c r="B222" s="2">
         <v>209</v>
@@ -18596,10 +18599,10 @@
         <v>141</v>
       </c>
       <c r="D222" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E222" s="26" t="s">
-        <v>1145</v>
+        <v>1149</v>
       </c>
       <c r="F222" s="6"/>
       <c r="G222" s="40" t="s">
@@ -18607,11 +18610,11 @@
       </c>
       <c r="H222" s="40" t="str">
         <f>CONCATENATE(D222,E222,F222)</f>
-        <v>E03</v>
+        <v>E08</v>
       </c>
       <c r="I222" s="5"/>
       <c r="J222" s="5" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="M222" s="19"/>
       <c r="N222" s="19"/>
@@ -18629,7 +18632,7 @@
         <v>998</v>
       </c>
       <c r="T222" s="5" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="U222" s="20" t="s">
         <v>141</v>
@@ -18645,36 +18648,36 @@
     <row r="223" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A223" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.03.a. - Homicide excluding legal intervention</v>
+        <v>....E.08.a. - Homicide excluding legal intervention</v>
       </c>
       <c r="B223" s="2"/>
       <c r="C223" s="31"/>
       <c r="D223" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E223" s="26" t="s">
-        <v>1145</v>
+        <v>1149</v>
       </c>
       <c r="F223" s="6" t="s">
         <v>1126</v>
       </c>
       <c r="G223" s="40" t="str">
         <f t="shared" si="23"/>
-        <v>cE03a</v>
+        <v>cE08a</v>
       </c>
       <c r="H223" s="40" t="str">
         <f t="shared" ref="H223:H225" si="24">CONCATENATE(D223,E223,F223)</f>
-        <v>E03a</v>
+        <v>E08a</v>
       </c>
       <c r="I223" s="5" t="s">
-        <v>1397</v>
+        <v>1395</v>
       </c>
       <c r="J223" s="5"/>
       <c r="K223" s="5" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
       <c r="L223" s="19" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
       <c r="M223" s="19"/>
       <c r="N223" s="19"/>
@@ -18684,7 +18687,7 @@
       <c r="R223" s="83"/>
       <c r="S223" s="83"/>
       <c r="T223" s="20" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="U223" s="46"/>
       <c r="V223" s="5"/>
@@ -18694,38 +18697,38 @@
     <row r="224" spans="1:24" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.03.b. - Legal intervention</v>
+        <v>....E.08.b. - Legal intervention</v>
       </c>
       <c r="B224" s="2"/>
       <c r="C224" s="31"/>
       <c r="D224" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E224" s="26" t="s">
-        <v>1145</v>
+        <v>1149</v>
       </c>
       <c r="F224" s="6" t="s">
         <v>1127</v>
       </c>
       <c r="G224" s="40" t="str">
         <f t="shared" si="23"/>
-        <v>cE03b</v>
+        <v>cE08b</v>
       </c>
       <c r="H224" s="40" t="str">
         <f t="shared" si="24"/>
-        <v>E03b</v>
+        <v>E08b</v>
       </c>
       <c r="I224" s="5" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
       <c r="J224" s="5" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="K224" s="5" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="L224" s="19" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="M224" s="19"/>
       <c r="N224" s="19"/>
@@ -18735,7 +18738,7 @@
       <c r="R224" s="83"/>
       <c r="S224" s="83"/>
       <c r="T224" s="20" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="U224" s="46"/>
       <c r="V224" s="5"/>
@@ -18745,7 +18748,7 @@
     <row r="225" spans="1:24" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A225" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.03.c. - Execution, War, Terroism</v>
+        <v>....E.08.c. - Execution, War, Terroism</v>
       </c>
       <c r="B225" s="2">
         <v>210</v>
@@ -18754,33 +18757,33 @@
         <v>142</v>
       </c>
       <c r="D225" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E225" s="26" t="s">
-        <v>1145</v>
+        <v>1149</v>
       </c>
       <c r="F225" s="6" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="G225" s="40" t="str">
         <f t="shared" si="23"/>
-        <v>cE03c</v>
+        <v>cE08c</v>
       </c>
       <c r="H225" s="40" t="str">
         <f t="shared" si="24"/>
-        <v>E03c</v>
+        <v>E08c</v>
       </c>
       <c r="I225" s="5" t="s">
-        <v>1399</v>
+        <v>1397</v>
       </c>
       <c r="J225" s="5" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="K225" s="5" t="s">
-        <v>1370</v>
+        <v>1368</v>
       </c>
       <c r="L225" s="49" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="M225" s="49"/>
       <c r="N225" s="49"/>
@@ -18794,7 +18797,7 @@
       <c r="R225" s="83"/>
       <c r="S225" s="83"/>
       <c r="T225" s="5" t="s">
-        <v>1374</v>
+        <v>1372</v>
       </c>
       <c r="U225" s="20" t="s">
         <v>142</v>
@@ -18806,7 +18809,7 @@
         <v>142</v>
       </c>
       <c r="X225" s="22" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="226" spans="1:24" ht="38.25" x14ac:dyDescent="0.25">
@@ -18815,36 +18818,36 @@
         <v/>
       </c>
       <c r="B226" s="77" t="s">
-        <v>1331</v>
+        <v>1401</v>
       </c>
       <c r="C226" s="16" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="D226" s="54" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="E226" s="55" t="s">
-        <v>1143</v>
+        <v>952</v>
       </c>
       <c r="G226" s="40" t="str">
         <f t="shared" si="23"/>
-        <v>cE01</v>
+        <v xml:space="preserve">cE </v>
       </c>
       <c r="H226" s="40"/>
       <c r="I226" s="48" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="J226" s="48" t="s">
+        <v>1268</v>
+      </c>
+      <c r="K226" s="16" t="s">
         <v>1269</v>
       </c>
-      <c r="K226" s="16" t="s">
+      <c r="L226" s="16" t="s">
         <v>1270</v>
       </c>
-      <c r="L226" s="16" t="s">
-        <v>1271</v>
-      </c>
       <c r="T226" s="48" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="227" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
@@ -18853,10 +18856,10 @@
         <v>...Z.01. - Symptoms, signs and ill-defined conditions, not elsewhere classified</v>
       </c>
       <c r="D227" s="56" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="E227" s="55" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="G227" s="40" t="str">
         <f t="shared" si="23"/>
@@ -18867,19 +18870,19 @@
         <v>Z01</v>
       </c>
       <c r="I227" s="48" t="s">
+        <v>1220</v>
+      </c>
+      <c r="J227" s="48" t="s">
         <v>1221</v>
       </c>
-      <c r="J227" s="48" t="s">
+      <c r="K227" s="16" t="s">
         <v>1222</v>
       </c>
-      <c r="K227" s="16" t="s">
+      <c r="L227" s="16" t="s">
+        <v>1251</v>
+      </c>
+      <c r="T227" s="48" t="s">
         <v>1223</v>
-      </c>
-      <c r="L227" s="16" t="s">
-        <v>1252</v>
-      </c>
-      <c r="T227" s="48" t="s">
-        <v>1224</v>
       </c>
     </row>
     <row r="228" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
@@ -18888,10 +18891,10 @@
         <v/>
       </c>
       <c r="D228" s="56" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="E228" s="55" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="G228" s="42" t="str">
         <f t="shared" si="23"/>
@@ -18899,19 +18902,19 @@
       </c>
       <c r="H228" s="40"/>
       <c r="I228" s="16" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="J228" s="48" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="K228" s="16" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="L228" s="16" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="T228" s="48" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="229" spans="1:24" x14ac:dyDescent="0.25">
@@ -18920,10 +18923,10 @@
         <v>...Z.02. - Unknown/Missing Value</v>
       </c>
       <c r="D229" s="56" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="E229" s="55" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="G229" s="43"/>
       <c r="H229" s="40" t="str">
@@ -18931,7 +18934,7 @@
         <v>Z02</v>
       </c>
       <c r="T229" s="48" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="230" spans="1:24" x14ac:dyDescent="0.25">
@@ -18940,10 +18943,10 @@
         <v>...Z.03. - Code does not map</v>
       </c>
       <c r="D230" s="56" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="E230" s="55" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="G230" s="43"/>
       <c r="H230" s="40" t="str">
@@ -18951,10 +18954,10 @@
         <v>Z03</v>
       </c>
       <c r="I230" s="16" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="T230" s="48" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="231" spans="1:24" x14ac:dyDescent="0.25">
@@ -18963,7 +18966,7 @@
         <v>..Z. - Unknown/Missing Value</v>
       </c>
       <c r="D231" s="56" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="G231" s="43"/>
       <c r="H231" s="40" t="str">
@@ -18971,7 +18974,7 @@
         <v>Z</v>
       </c>
       <c r="T231" s="48" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="232" spans="1:24" x14ac:dyDescent="0.25">
@@ -18980,10 +18983,10 @@
         <v>...D.99. - Other Chronic Conditions</v>
       </c>
       <c r="D232" s="56" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="E232" s="55" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="G232" s="43"/>
       <c r="H232" s="40" t="str">
@@ -18991,7 +18994,7 @@
         <v>D99</v>
       </c>
       <c r="T232" s="48" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
     </row>
   </sheetData>
@@ -19222,24 +19225,24 @@
   <sheetData>
     <row r="11" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="70" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="D11" s="71" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="E11" s="71" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="12" spans="3:5" ht="135.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="72" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D12" s="73" t="s">
         <v>1317</v>
       </c>
-      <c r="D12" s="73" t="s">
+      <c r="E12" s="73" t="s">
         <v>1318</v>
-      </c>
-      <c r="E12" s="73" t="s">
-        <v>1319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new 2018 dataset and misc clean up
</commit_message>
<xml_diff>
--- a/myCBD/myInfo/gbd.ICD.Map.xlsx
+++ b/myCBD/myInfo/gbd.ICD.Map.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr autoCompressPictures="0" defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0.CBD\myCBD\myInfo\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24240" windowHeight="10935"/>
   </bookViews>
@@ -19,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">main!$A$1:$X$225</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -36,7 +31,7 @@
     <author>Dauphine, David (CDPH-CHSI)</author>
   </authors>
   <commentList>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -60,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C57" authorId="1" shapeId="0">
+    <comment ref="C57" authorId="1">
       <text>
         <r>
           <rPr>
@@ -84,7 +79,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P126" authorId="2" shapeId="0">
+    <comment ref="P126" authorId="2">
       <text>
         <r>
           <rPr>
@@ -113,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2869" uniqueCount="1402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2860" uniqueCount="1418">
   <si>
     <t>I. Communicable, maternal, perinatal and nutritional conditions</t>
   </si>
@@ -4339,9 +4334,6 @@
     <t>Y35[0-4]|Y35[6-9]|Y890</t>
   </si>
   <si>
-    <t>Execution, War, Terroism</t>
-  </si>
-  <si>
     <t>W32-W34.9</t>
   </si>
   <si>
@@ -4373,12 +4365,6 @@
     <t>2. Non-SA Poisonings</t>
   </si>
   <si>
-    <t>X42|X44</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> X42, X44</t>
-  </si>
-  <si>
     <t>DELETED X42 and X44 per CDPH review (1/9/2019) - to Substance Use - associated poisonings;</t>
   </si>
   <si>
@@ -4388,19 +4374,10 @@
     <t>F1[3,6,8,9]|P044</t>
   </si>
   <si>
-    <t>X4[0,1,3,6-9]</t>
-  </si>
-  <si>
-    <t>X40, X41, X43, X46-X49</t>
-  </si>
-  <si>
     <t>E.2. Substance use disorders</t>
   </si>
   <si>
     <t>Substance use disorders</t>
-  </si>
-  <si>
-    <t>Substance use-associated poisonings</t>
   </si>
   <si>
     <r>
@@ -4463,16 +4440,82 @@
     <t>Added P044  ; as above moved X41 to Poisonings (non-substance)</t>
   </si>
   <si>
-    <t>Poisonings (non-substance use)</t>
-  </si>
-  <si>
     <t>INCLUDED ALL INJURY but not elsewhere</t>
+  </si>
+  <si>
+    <t>Drug poisonings</t>
+  </si>
+  <si>
+    <t>Poisonings (non-drug)</t>
+  </si>
+  <si>
+    <t>(moved x40,x41, and x 43 Up one</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> X40- X44</t>
+  </si>
+  <si>
+    <t>X46-X49</t>
+  </si>
+  <si>
+    <t>X4[6-9]</t>
+  </si>
+  <si>
+    <t>Gonorrhea</t>
+  </si>
+  <si>
+    <t>Diarrheal diseases</t>
+  </si>
+  <si>
+    <t>Maternal hemorrhage</t>
+  </si>
+  <si>
+    <t>Esophagus cancer</t>
+  </si>
+  <si>
+    <t>Leukemia</t>
+  </si>
+  <si>
+    <t>Autism and Asperger syndrome</t>
+  </si>
+  <si>
+    <t>Childhood behavioral disorders</t>
+  </si>
+  <si>
+    <t>Other mental and behavioral disorders</t>
+  </si>
+  <si>
+    <t>Ischemic heart disease</t>
+  </si>
+  <si>
+    <t>Chronic kidney disease due to diabetes</t>
+  </si>
+  <si>
+    <t>Execution, War, Terrorism</t>
+  </si>
+  <si>
+    <t>Obstructed labor</t>
+  </si>
+  <si>
+    <t>Iron-deficiency anemia</t>
+  </si>
+  <si>
+    <t>Nasopharynx</t>
+  </si>
+  <si>
+    <t>Gallbladder and biliary tract cancer</t>
+  </si>
+  <si>
+    <t>Other haemoglobinopathies and hemolytic anemias</t>
+  </si>
+  <si>
+    <t>X4[0-4]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="###0.;###0."/>
   </numFmts>
@@ -5157,7 +5200,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -5192,7 +5235,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -6032,7 +6075,7 @@
         <v>1047</v>
       </c>
       <c r="T11" s="5" t="s">
-        <v>149</v>
+        <v>1401</v>
       </c>
       <c r="U11" s="20" t="s">
         <v>6</v>
@@ -6386,7 +6429,7 @@
         <v>1059</v>
       </c>
       <c r="T17" s="5" t="s">
-        <v>155</v>
+        <v>1402</v>
       </c>
       <c r="U17" s="20" t="s">
         <v>10</v>
@@ -8676,7 +8719,7 @@
         <v>1066</v>
       </c>
       <c r="T57" s="5" t="s">
-        <v>193</v>
+        <v>1403</v>
       </c>
       <c r="U57" s="20" t="s">
         <v>33</v>
@@ -8872,7 +8915,7 @@
         <v>1065</v>
       </c>
       <c r="T60" s="5" t="s">
-        <v>196</v>
+        <v>1412</v>
       </c>
       <c r="U60" s="20" t="s">
         <v>36</v>
@@ -9583,7 +9626,7 @@
         <v>1033</v>
       </c>
       <c r="T72" s="5" t="s">
-        <v>208</v>
+        <v>1413</v>
       </c>
       <c r="U72" s="20" t="s">
         <v>48</v>
@@ -9688,7 +9731,7 @@
       </c>
       <c r="Q74" s="59"/>
       <c r="R74" s="86" t="s">
-        <v>1393</v>
+        <v>1387</v>
       </c>
       <c r="S74" s="83" t="s">
         <v>557</v>
@@ -9977,7 +10020,7 @@
         <v>1087</v>
       </c>
       <c r="T79" s="5" t="s">
-        <v>214</v>
+        <v>1414</v>
       </c>
       <c r="U79" s="50" t="s">
         <v>896</v>
@@ -10053,7 +10096,7 @@
     <row r="81" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A81" s="44" t="str">
         <f t="shared" si="5"/>
-        <v>...B.02. - Oesophagus cancer</v>
+        <v>...B.02. - Esophagus cancer</v>
       </c>
       <c r="B81" s="2">
         <v>75</v>
@@ -10104,7 +10147,7 @@
         <v>1089</v>
       </c>
       <c r="T81" s="5" t="s">
-        <v>216</v>
+        <v>1404</v>
       </c>
       <c r="U81" s="50" t="s">
         <v>53</v>
@@ -11329,7 +11372,7 @@
         <v>1075</v>
       </c>
       <c r="T100" s="5" t="s">
-        <v>897</v>
+        <v>1415</v>
       </c>
       <c r="U100" s="20" t="s">
         <v>707</v>
@@ -11788,7 +11831,7 @@
     <row r="108" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A108" s="44" t="str">
         <f t="shared" si="5"/>
-        <v>...B.17. - Leukaemia</v>
+        <v>...B.17. - Leukemia</v>
       </c>
       <c r="B108" s="2">
         <v>101</v>
@@ -11835,7 +11878,7 @@
         <v>1030</v>
       </c>
       <c r="T108" s="5" t="s">
-        <v>235</v>
+        <v>1405</v>
       </c>
       <c r="U108" s="20" t="s">
         <v>715</v>
@@ -12271,7 +12314,7 @@
         <v>1105</v>
       </c>
       <c r="T115" s="5" t="s">
-        <v>242</v>
+        <v>1416</v>
       </c>
       <c r="U115" s="5" t="s">
         <v>719</v>
@@ -12454,7 +12497,7 @@
       </c>
       <c r="B119" s="2"/>
       <c r="C119" s="32" t="s">
-        <v>1390</v>
+        <v>1385</v>
       </c>
       <c r="D119" s="6" t="s">
         <v>1140</v>
@@ -12480,7 +12523,7 @@
       <c r="R119" s="83"/>
       <c r="S119" s="83"/>
       <c r="T119" s="2" t="s">
-        <v>1391</v>
+        <v>1386</v>
       </c>
       <c r="U119" s="20"/>
       <c r="V119" s="2" t="s">
@@ -12964,14 +13007,14 @@
         <v>D04b</v>
       </c>
       <c r="I128" s="79" t="s">
-        <v>1385</v>
+        <v>1382</v>
       </c>
       <c r="J128" s="5"/>
       <c r="K128" s="5" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="L128" s="49" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="M128" s="49"/>
       <c r="N128" s="49"/>
@@ -13211,16 +13254,16 @@
       </c>
       <c r="H132" s="40"/>
       <c r="I132" s="79" t="s">
-        <v>1399</v>
+        <v>1393</v>
       </c>
       <c r="J132" s="5" t="s">
         <v>1159</v>
       </c>
       <c r="K132" s="5" t="s">
-        <v>1386</v>
+        <v>1383</v>
       </c>
       <c r="L132" s="19" t="s">
-        <v>1387</v>
+        <v>1384</v>
       </c>
       <c r="M132" s="19"/>
       <c r="N132" s="19"/>
@@ -13412,7 +13455,7 @@
       <c r="R135" s="83"/>
       <c r="S135" s="83"/>
       <c r="T135" s="5" t="s">
-        <v>914</v>
+        <v>1406</v>
       </c>
       <c r="U135" s="5" t="s">
         <v>918</v>
@@ -13461,7 +13504,7 @@
       <c r="R136" s="83"/>
       <c r="S136" s="83"/>
       <c r="T136" s="5" t="s">
-        <v>915</v>
+        <v>1407</v>
       </c>
       <c r="U136" s="5" t="s">
         <v>74</v>
@@ -13685,7 +13728,7 @@
       <c r="R140" s="83"/>
       <c r="S140" s="83"/>
       <c r="T140" s="5" t="s">
-        <v>253</v>
+        <v>1408</v>
       </c>
       <c r="U140" s="20" t="s">
         <v>76</v>
@@ -14820,7 +14863,7 @@
     <row r="160" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A160" s="44" t="str">
         <f t="shared" si="12"/>
-        <v>...C.02. - Ischaemic heart disease</v>
+        <v>...C.02. - Ischemic heart disease</v>
       </c>
       <c r="B160" s="2">
         <v>150</v>
@@ -14871,7 +14914,7 @@
         <v>1029</v>
       </c>
       <c r="T160" s="5" t="s">
-        <v>273</v>
+        <v>1409</v>
       </c>
       <c r="U160" s="50" t="s">
         <v>96</v>
@@ -16198,7 +16241,7 @@
     <row r="182" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A182" s="44" t="str">
         <f t="shared" si="12"/>
-        <v>....D.10.b. - Chronic kidney diesease due to diabetes</v>
+        <v>....D.10.b. - Chronic kidney disease due to diabetes</v>
       </c>
       <c r="B182" s="2">
         <v>171</v>
@@ -16249,7 +16292,7 @@
         <v>2504</v>
       </c>
       <c r="T182" s="5" t="s">
-        <v>926</v>
+        <v>1410</v>
       </c>
       <c r="U182" s="5" t="s">
         <v>928</v>
@@ -17772,7 +17815,7 @@
       </c>
       <c r="Q208" s="62"/>
       <c r="R208" s="86" t="s">
-        <v>1394</v>
+        <v>1388</v>
       </c>
       <c r="S208" s="83" t="s">
         <v>654</v>
@@ -17851,7 +17894,7 @@
     <row r="210" spans="1:24" ht="36" x14ac:dyDescent="0.25">
       <c r="A210" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.01. . - Road injury</v>
+        <v>...E.01. - Road injury</v>
       </c>
       <c r="B210" s="2">
         <v>199</v>
@@ -17865,16 +17908,14 @@
       <c r="E210" s="26" t="s">
         <v>1142</v>
       </c>
-      <c r="F210" s="88" t="s">
-        <v>952</v>
-      </c>
+      <c r="F210" s="88"/>
       <c r="G210" s="40" t="str">
         <f t="shared" ref="G210:G219" si="21">CONCATENATE("c",D210,E210,F210)</f>
-        <v xml:space="preserve">cE01 </v>
+        <v>cE01</v>
       </c>
       <c r="H210" s="40" t="str">
         <f>CONCATENATE(D210,E210,F210)</f>
-        <v xml:space="preserve">E01 </v>
+        <v>E01</v>
       </c>
       <c r="I210" s="5" t="s">
         <v>1234</v>
@@ -17917,14 +17958,14 @@
       </c>
       <c r="X210" s="2"/>
     </row>
-    <row r="211" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:24" ht="15" x14ac:dyDescent="0.25">
       <c r="A211" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.02. . - Substance use-associated poisonings</v>
+        <v>...E.02. - Drug poisonings</v>
       </c>
       <c r="B211" s="2"/>
       <c r="C211" s="31" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
       <c r="D211" s="6" t="s">
         <v>1141</v>
@@ -17932,24 +17973,24 @@
       <c r="E211" s="26" t="s">
         <v>1143</v>
       </c>
-      <c r="F211" s="88" t="s">
-        <v>952</v>
-      </c>
+      <c r="F211" s="88"/>
       <c r="G211" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE02 </v>
+        <v>cE02</v>
       </c>
       <c r="H211" s="40" t="str">
         <f t="shared" ref="H211:H212" si="22">CONCATENATE(D211,E211,F211)</f>
-        <v xml:space="preserve">E02 </v>
-      </c>
-      <c r="I211" s="5"/>
+        <v>E02</v>
+      </c>
+      <c r="I211" t="s">
+        <v>952</v>
+      </c>
       <c r="J211" s="5"/>
       <c r="K211" s="79" t="s">
-        <v>1384</v>
+        <v>1398</v>
       </c>
       <c r="L211" s="80" t="s">
-        <v>1383</v>
+        <v>1417</v>
       </c>
       <c r="M211" s="19"/>
       <c r="N211" s="19"/>
@@ -17959,23 +18000,23 @@
       <c r="R211" s="83"/>
       <c r="S211" s="83"/>
       <c r="T211" s="5" t="s">
-        <v>1392</v>
+        <v>1395</v>
       </c>
       <c r="U211" s="20"/>
       <c r="V211" s="5"/>
       <c r="W211" s="45"/>
       <c r="X211" s="2"/>
     </row>
-    <row r="212" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:24" ht="51" x14ac:dyDescent="0.25">
       <c r="A212" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.03. . - Poisonings (non-substance use)</v>
+        <v>...E.03. - Poisonings (non-drug)</v>
       </c>
       <c r="B212" s="2">
         <v>200</v>
       </c>
       <c r="C212" s="31" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
       <c r="D212" s="6" t="s">
         <v>1141</v>
@@ -17983,24 +18024,24 @@
       <c r="E212" s="26" t="s">
         <v>1144</v>
       </c>
-      <c r="F212" s="88" t="s">
-        <v>952</v>
-      </c>
+      <c r="F212" s="88"/>
       <c r="G212" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE03 </v>
+        <v>cE03</v>
       </c>
       <c r="H212" s="40" t="str">
         <f t="shared" si="22"/>
-        <v xml:space="preserve">E03 </v>
+        <v>E03</v>
       </c>
       <c r="I212" s="5"/>
-      <c r="J212" s="5"/>
+      <c r="J212" s="5" t="s">
+        <v>1397</v>
+      </c>
       <c r="K212" s="79" t="s">
-        <v>1389</v>
+        <v>1399</v>
       </c>
       <c r="L212" s="81" t="s">
-        <v>1388</v>
+        <v>1400</v>
       </c>
       <c r="M212" s="49"/>
       <c r="N212" s="49"/>
@@ -18018,7 +18059,7 @@
         <v>1006</v>
       </c>
       <c r="T212" s="5" t="s">
-        <v>1400</v>
+        <v>1396</v>
       </c>
       <c r="U212" s="20" t="s">
         <v>135</v>
@@ -18034,7 +18075,7 @@
     <row r="213" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A213" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.04. . - Falls</v>
+        <v>...E.04. - Falls</v>
       </c>
       <c r="B213" s="2">
         <v>201</v>
@@ -18048,16 +18089,14 @@
       <c r="E213" s="26" t="s">
         <v>1145</v>
       </c>
-      <c r="F213" s="88" t="s">
-        <v>952</v>
-      </c>
+      <c r="F213" s="88"/>
       <c r="G213" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE04 </v>
+        <v>cE04</v>
       </c>
       <c r="H213" s="40" t="str">
         <f>CONCATENATE(D213,E213,F213)</f>
-        <v xml:space="preserve">E04 </v>
+        <v>E04</v>
       </c>
       <c r="I213" s="5" t="s">
         <v>952</v>
@@ -18115,12 +18154,10 @@
       <c r="E214" s="26" t="s">
         <v>1146</v>
       </c>
-      <c r="F214" s="6" t="s">
-        <v>952</v>
-      </c>
+      <c r="F214" s="6"/>
       <c r="G214" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE05 </v>
+        <v>cE05</v>
       </c>
       <c r="H214" s="40"/>
       <c r="K214" s="5" t="s">
@@ -18175,12 +18212,10 @@
       <c r="E215" s="26" t="s">
         <v>1146</v>
       </c>
-      <c r="F215" s="6" t="s">
-        <v>952</v>
-      </c>
+      <c r="F215" s="6"/>
       <c r="G215" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE05 </v>
+        <v>cE05</v>
       </c>
       <c r="H215" s="40"/>
       <c r="I215" s="5"/>
@@ -18237,21 +18272,19 @@
       <c r="E216" s="26" t="s">
         <v>1146</v>
       </c>
-      <c r="F216" s="6" t="s">
-        <v>952</v>
-      </c>
+      <c r="F216" s="6"/>
       <c r="G216" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE05 </v>
+        <v>cE05</v>
       </c>
       <c r="H216" s="40"/>
       <c r="I216" s="5"/>
       <c r="J216" s="5"/>
       <c r="K216" s="5" t="s">
-        <v>1377</v>
+        <v>1376</v>
       </c>
       <c r="L216" s="49" t="s">
-        <v>1379</v>
+        <v>1378</v>
       </c>
       <c r="M216" s="49"/>
       <c r="N216" s="49"/>
@@ -18285,11 +18318,11 @@
     <row r="217" spans="1:24" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A217" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.05. . - Accidental Firearm</v>
+        <v/>
       </c>
       <c r="B217" s="2"/>
       <c r="C217" s="31" t="s">
-        <v>1378</v>
+        <v>1377</v>
       </c>
       <c r="D217" s="6" t="s">
         <v>1141</v>
@@ -18297,27 +18330,23 @@
       <c r="E217" s="26" t="s">
         <v>1146</v>
       </c>
-      <c r="F217" s="6" t="s">
-        <v>952</v>
-      </c>
+      <c r="F217" s="6"/>
       <c r="G217" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE05 </v>
-      </c>
-      <c r="H217" s="40" t="s">
-        <v>952</v>
-      </c>
+        <v>cE05</v>
+      </c>
+      <c r="H217" s="40"/>
       <c r="I217" s="5" t="s">
-        <v>1376</v>
+        <v>1375</v>
       </c>
       <c r="J217" s="5" t="s">
         <v>1211</v>
       </c>
       <c r="K217" s="5" t="s">
+        <v>1372</v>
+      </c>
+      <c r="L217" s="49" t="s">
         <v>1373</v>
-      </c>
-      <c r="L217" s="49" t="s">
-        <v>1374</v>
       </c>
       <c r="M217" s="49"/>
       <c r="N217" s="49"/>
@@ -18327,7 +18356,7 @@
       <c r="R217" s="83"/>
       <c r="S217" s="83"/>
       <c r="T217" s="5" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="U217" s="20"/>
       <c r="V217" s="5"/>
@@ -18351,12 +18380,10 @@
       <c r="E218" s="26" t="s">
         <v>1146</v>
       </c>
-      <c r="F218" s="6" t="s">
-        <v>952</v>
-      </c>
+      <c r="F218" s="6"/>
       <c r="G218" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE05 </v>
+        <v>cE05</v>
       </c>
       <c r="H218" s="40"/>
       <c r="I218" s="5" t="s">
@@ -18399,7 +18426,7 @@
     <row r="219" spans="1:24" ht="33" x14ac:dyDescent="0.25">
       <c r="A219" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.05. . - Other unintentional injuries</v>
+        <v>...E.05. - Other unintentional injuries</v>
       </c>
       <c r="B219" s="2">
         <v>206</v>
@@ -18413,19 +18440,17 @@
       <c r="E219" s="26" t="s">
         <v>1146</v>
       </c>
-      <c r="F219" s="6" t="s">
-        <v>952</v>
-      </c>
+      <c r="F219" s="6"/>
       <c r="G219" s="40" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">cE05 </v>
+        <v>cE05</v>
       </c>
       <c r="H219" s="40" t="str">
         <f>CONCATENATE(D219,E219,F219)</f>
-        <v xml:space="preserve">E05 </v>
+        <v>E05</v>
       </c>
       <c r="I219" s="5" t="s">
-        <v>1398</v>
+        <v>1392</v>
       </c>
       <c r="J219" s="5" t="s">
         <v>1253</v>
@@ -18666,11 +18691,11 @@
         <v>cE08a</v>
       </c>
       <c r="H223" s="40" t="str">
-        <f t="shared" ref="H223:H225" si="24">CONCATENATE(D223,E223,F223)</f>
+        <f t="shared" ref="H223:H226" si="24">CONCATENATE(D223,E223,F223)</f>
         <v>E08a</v>
       </c>
       <c r="I223" s="5" t="s">
-        <v>1395</v>
+        <v>1389</v>
       </c>
       <c r="J223" s="5"/>
       <c r="K223" s="5" t="s">
@@ -18719,7 +18744,7 @@
         <v>E08b</v>
       </c>
       <c r="I224" s="5" t="s">
-        <v>1396</v>
+        <v>1390</v>
       </c>
       <c r="J224" s="5" t="s">
         <v>1211</v>
@@ -18748,7 +18773,7 @@
     <row r="225" spans="1:24" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A225" s="44" t="str">
         <f t="shared" si="19"/>
-        <v>....E.08.c. - Execution, War, Terroism</v>
+        <v>....E.08.c. - Execution, War, Terrorism</v>
       </c>
       <c r="B225" s="2">
         <v>210</v>
@@ -18774,7 +18799,7 @@
         <v>E08c</v>
       </c>
       <c r="I225" s="5" t="s">
-        <v>1397</v>
+        <v>1391</v>
       </c>
       <c r="J225" s="5" t="s">
         <v>1236</v>
@@ -18797,7 +18822,7 @@
       <c r="R225" s="83"/>
       <c r="S225" s="83"/>
       <c r="T225" s="5" t="s">
-        <v>1372</v>
+        <v>1411</v>
       </c>
       <c r="U225" s="20" t="s">
         <v>142</v>
@@ -18815,10 +18840,10 @@
     <row r="226" spans="1:24" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A226" s="44" t="str">
         <f t="shared" si="19"/>
-        <v/>
+        <v>...E.99. - Injuries of unknown intent (e.g., unintentional or self-harm), including overdoses and deaths by firearm</v>
       </c>
       <c r="B226" s="77" t="s">
-        <v>1401</v>
+        <v>1394</v>
       </c>
       <c r="C226" s="16" t="s">
         <v>1275</v>
@@ -18827,13 +18852,16 @@
         <v>1141</v>
       </c>
       <c r="E226" s="55" t="s">
-        <v>952</v>
+        <v>1224</v>
       </c>
       <c r="G226" s="40" t="str">
         <f t="shared" si="23"/>
-        <v xml:space="preserve">cE </v>
-      </c>
-      <c r="H226" s="40"/>
+        <v>cE99</v>
+      </c>
+      <c r="H226" s="40" t="str">
+        <f t="shared" si="24"/>
+        <v>E99</v>
+      </c>
       <c r="I226" s="48" t="s">
         <v>1252</v>
       </c>

</xml_diff>